<commit_message>
Fixed First year and grad checker to no longer produce incorect results, added code to start multiple imputation toadress missing variables
</commit_message>
<xml_diff>
--- a/Variable_Check.xlsx
+++ b/Variable_Check.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="84">
   <si>
     <t>Variable</t>
   </si>
@@ -172,49 +172,52 @@
     <t>dr_ft_frst_men_forgn_v, dr_ft_frst_wmen_forgn_v</t>
   </si>
   <si>
+    <t>ma_ft_men_all_races_v, ma_ft_wmen_all_races_v</t>
+  </si>
+  <si>
+    <t>ma_ft_tot_black_v, ma_ft_tot_indian_v, ma_ft_tot_asian_v, ma_ft_tot_pacific_v, ma_ft_tot_white_v, ma_ft_tot_hisp_v, ma_ft_tot_multi_v, ma_ft_tot_unk_v, ma_ft_tot_forgn_v</t>
+  </si>
+  <si>
+    <t>ma_ft_frst_men_black_v, ma_ft_frst_wmen_black_v</t>
+  </si>
+  <si>
+    <t>ma_ft_frst_men_indian_v, ma_ft_frst_wmen_indian_v</t>
+  </si>
+  <si>
+    <t>ma_ft_frst_men_asian_v, ma_ft_frst_wmen_asian_v</t>
+  </si>
+  <si>
+    <t>ma_ft_frst_men_pacific_v, ma_ft_frst_wmen_pacific_v</t>
+  </si>
+  <si>
+    <t>ma_ft_frst_men_white_v, ma_ft_frst_wmen_white_v</t>
+  </si>
+  <si>
+    <t>ma_ft_frst_men_hisp_v, ma_ft_frst_wmen_hisp_v</t>
+  </si>
+  <si>
+    <t>ma_ft_frst_men_multi_v, ma_ft_frst_wmen_multi_v</t>
+  </si>
+  <si>
+    <t>ma_ft_frst_men_unk_v, ma_ft_frst_wmen_unk_v</t>
+  </si>
+  <si>
+    <t>ma_ft_frst_men_forgn_v, ma_ft_frst_wmen_forgn_v</t>
+  </si>
+  <si>
+    <t>ma_ft_frst_men_black_v, ma_ft_frst_men_indian_v, ma_ft_frst_men_asian_v, ma_ft_frst_men_pacific_v, ma_ft_frst_men_white_v, ma_ft_frst_men_hisp_v, ma_ft_frst_men_multi_v, ma_ft_frst_men_unk_v, ma_ft_frst_men_forgn_v</t>
+  </si>
+  <si>
+    <t>dr_ft_frst_men_black_v, dr_ft_frst_men_indian_v, dr_ft_frst_men_asian_v, dr_ft_frst_men_pacific_v, dr_ft_frst_men_white_v, dr_ft_frst_men_hisp_v, dr_ft_frst_men_multi_v, dr_ft_frst_men_unk_v, dr_ft_frst_men_forgn_v</t>
+  </si>
+  <si>
+    <t>ma_ft_frst_wmen_black_v, ma_ft_frst_wmen_indian_v, ma_ft_frst_wmen_asian_v, ma_ft_frst_wmen_pacific_v, ma_ft_frst_wmen_white_v, ma_ft_frst_wmen_hisp_v, ma_ft_frst_wmen_multi_v, ma_ft_frst_wmen_unk_v, ma_ft_frst_wmen_forgn_v</t>
+  </si>
+  <si>
+    <t>dr_ft_frst_wmen_black_v, dr_ft_frst_wmen_indian_v, dr_ft_frst_wmen_asian_v, dr_ft_frst_wmen_pacific_v, dr_ft_frst_wmen_white_v, dr_ft_frst_wmen_hisp_v, dr_ft_frst_wmen_multi_v, dr_ft_frst_wmen_unk_v, dr_ft_frst_wmen_forgn_v</t>
+  </si>
+  <si>
     <t>ma_ft_frst_men_all_races_v, ma_ft_frst_wmen_all_races_v</t>
-  </si>
-  <si>
-    <t>ma_ft_tot_black_v, ma_ft_tot_indian_v, ma_ft_tot_asian_v, ma_ft_tot_pacific_v, ma_ft_tot_white_v, ma_ft_tot_hisp_v, ma_ft_tot_multi_v, ma_ft_tot_unk_v, ma_ft_tot_forgn_v</t>
-  </si>
-  <si>
-    <t>ma_ft_frst_men_black_v, ma_ft_frst_wmen_black_v</t>
-  </si>
-  <si>
-    <t>ma_ft_frst_men_indian_v, ma_ft_frst_wmen_indian_v</t>
-  </si>
-  <si>
-    <t>ma_ft_frst_men_asian_v, ma_ft_frst_wmen_asian_v</t>
-  </si>
-  <si>
-    <t>ma_ft_frst_men_pacific_v, ma_ft_frst_wmen_pacific_v</t>
-  </si>
-  <si>
-    <t>ma_ft_frst_men_white_v, ma_ft_frst_wmen_white_v</t>
-  </si>
-  <si>
-    <t>ma_ft_frst_men_hisp_v, ma_ft_frst_wmen_hisp_v</t>
-  </si>
-  <si>
-    <t>ma_ft_frst_men_multi_v, ma_ft_frst_wmen_multi_v</t>
-  </si>
-  <si>
-    <t>ma_ft_frst_men_unk_v, ma_ft_frst_wmen_unk_v</t>
-  </si>
-  <si>
-    <t>ma_ft_frst_men_forgn_v, ma_ft_frst_wmen_forgn_v</t>
-  </si>
-  <si>
-    <t>ma_ft_frst_men_black_v, ma_ft_frst_men_indian_v, ma_ft_frst_men_asian_v, ma_ft_frst_men_pacific_v, ma_ft_frst_men_white_v, ma_ft_frst_men_hisp_v, ma_ft_frst_men_multi_v, ma_ft_frst_men_unk_v, ma_ft_frst_men_forgn_v</t>
-  </si>
-  <si>
-    <t>dr_ft_frst_men_black_v, dr_ft_frst_men_indian_v, dr_ft_frst_men_asian_v, dr_ft_frst_men_pacific_v, dr_ft_frst_men_white_v, dr_ft_frst_men_hisp_v, dr_ft_frst_men_multi_v, dr_ft_frst_men_unk_v, dr_ft_frst_men_forgn_v</t>
-  </si>
-  <si>
-    <t>ma_ft_frst_wmen_black_v, ma_ft_frst_wmen_indian_v, ma_ft_frst_wmen_asian_v, ma_ft_frst_wmen_pacific_v, ma_ft_frst_wmen_white_v, ma_ft_frst_wmen_hisp_v, ma_ft_frst_wmen_multi_v, ma_ft_frst_wmen_unk_v, ma_ft_frst_wmen_forgn_v</t>
-  </si>
-  <si>
-    <t>dr_ft_frst_wmen_black_v, dr_ft_frst_wmen_indian_v, dr_ft_frst_wmen_asian_v, dr_ft_frst_wmen_pacific_v, dr_ft_frst_wmen_white_v, dr_ft_frst_wmen_hisp_v, dr_ft_frst_wmen_multi_v, dr_ft_frst_wmen_unk_v, dr_ft_frst_wmen_forgn_v</t>
   </si>
   <si>
     <t>ma_ft_men_black_v, ma_ft_men_indian_v, ma_ft_men_asian_v, ma_ft_men_pacific_v, ma_ft_men_white_v, ma_ft_men_hisp_v, ma_ft_men_multi_v, ma_ft_men_unk_v, ma_ft_men_forgn_v</t>
@@ -654,7 +657,7 @@
         <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -671,7 +674,7 @@
         <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -688,7 +691,7 @@
         <v>42</v>
       </c>
       <c r="D4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -705,7 +708,7 @@
         <v>43</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -722,7 +725,7 @@
         <v>44</v>
       </c>
       <c r="D6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -739,7 +742,7 @@
         <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -756,7 +759,7 @@
         <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -773,7 +776,7 @@
         <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -790,7 +793,7 @@
         <v>48</v>
       </c>
       <c r="D10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -807,7 +810,7 @@
         <v>49</v>
       </c>
       <c r="D11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -824,7 +827,7 @@
         <v>50</v>
       </c>
       <c r="D12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -841,7 +844,7 @@
         <v>51</v>
       </c>
       <c r="D13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -861,7 +864,7 @@
         <v>82</v>
       </c>
       <c r="F14">
-        <v>5911</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -875,7 +878,7 @@
         <v>53</v>
       </c>
       <c r="D15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -892,7 +895,7 @@
         <v>54</v>
       </c>
       <c r="D16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -909,7 +912,7 @@
         <v>55</v>
       </c>
       <c r="D17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -926,7 +929,7 @@
         <v>56</v>
       </c>
       <c r="D18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -943,7 +946,7 @@
         <v>57</v>
       </c>
       <c r="D19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -960,7 +963,7 @@
         <v>58</v>
       </c>
       <c r="D20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -977,7 +980,7 @@
         <v>59</v>
       </c>
       <c r="D21" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -994,7 +997,7 @@
         <v>60</v>
       </c>
       <c r="D22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -1011,7 +1014,7 @@
         <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -1028,7 +1031,7 @@
         <v>62</v>
       </c>
       <c r="D24" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1045,7 +1048,7 @@
         <v>63</v>
       </c>
       <c r="D25" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1062,7 +1065,7 @@
         <v>64</v>
       </c>
       <c r="D26" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -1079,7 +1082,7 @@
         <v>65</v>
       </c>
       <c r="D27" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -1096,7 +1099,7 @@
         <v>66</v>
       </c>
       <c r="D28" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F28">
         <v>0</v>
@@ -1110,10 +1113,10 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="D29" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F29">
         <v>0</v>
@@ -1127,10 +1130,10 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F30">
         <v>0</v>
@@ -1144,10 +1147,10 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D31" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F31">
         <v>0</v>
@@ -1161,10 +1164,10 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D32" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F32">
         <v>0</v>
@@ -1178,10 +1181,10 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D33" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F33">
         <v>0</v>
@@ -1195,10 +1198,10 @@
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D34" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F34">
         <v>0</v>
@@ -1212,13 +1215,13 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D35" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F35">
-        <v>1499</v>
+        <v>132</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -1229,13 +1232,13 @@
         <v>2</v>
       </c>
       <c r="C36" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D36" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F36">
-        <v>239</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -1246,13 +1249,13 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D37" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F37">
-        <v>1216</v>
+        <v>41</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -1263,13 +1266,13 @@
         <v>2</v>
       </c>
       <c r="C38" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D38" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F38">
-        <v>232</v>
+        <v>24</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -1280,13 +1283,13 @@
         <v>1</v>
       </c>
       <c r="C39" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D39" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F39">
-        <v>1084</v>
+        <v>214</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -1297,13 +1300,13 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D40" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F40">
-        <v>388</v>
+        <v>61</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -1314,13 +1317,13 @@
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D41" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F41">
-        <v>50051</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -1331,13 +1334,13 @@
         <v>2</v>
       </c>
       <c r="C42" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D42" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F42">
-        <v>31006</v>
+        <v>67</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -1348,13 +1351,13 @@
         <v>3</v>
       </c>
       <c r="C43" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D43" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F43">
-        <v>50009</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>